<commit_message>
Add 947-953 11th St OM and re-underwrite from its rent roll and expenses; rebuild public and Shawn Mangoli pages
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/files/03-947-953-11th-st.xlsx
+++ b/files/03-947-953-11th-st.xlsx
@@ -8,17 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\iniculete\LAAA-Deploys\onmarket\files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{5A36D8F5-6750-46C0-9272-C97435FBB704}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{93D6BE28-8CD9-42FE-8D18-22C275D06059}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{E859AC3A-34D8-4D3A-8146-67E63EC8F48F}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{26B3E24F-726B-438B-AD7A-01605760F0D5}"/>
   </bookViews>
   <sheets>
     <sheet name="Assumptions" sheetId="1" r:id="rId1"/>
     <sheet name="03 947-953 11th St" sheetId="2" r:id="rId2"/>
   </sheets>
-  <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="1">'03 947-953 11th St'!$A$1:$N$78</definedName>
-  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -43,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="153" uniqueCount="142">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="154" uniqueCount="144">
   <si>
     <t>LAAA UNDERWRITING BENCHMARKS (edit here; every deal tab reads these)</t>
   </si>
@@ -195,10 +192,10 @@
     <t>LoopNet listing</t>
   </si>
   <si>
-    <t>Data pulled 9/17/2026 from LoopNet public listing</t>
-  </si>
-  <si>
-    <t>NOTE: 80% occupied per LoopNet</t>
+    <t>Data pulled 9/17/2026 from LoopNet public listing + rent roll and expenses read from the listing broker's OM (Equity Union Commercial (The Appel Group), Eliyahu Appel, undated, sale comps through May 2026)</t>
+  </si>
+  <si>
+    <t>NOTE: 80% occupied per LoopNet | OM: Mills Act: existing recorded Mills Act contract; OM carries property taxes at $36,816 (current bill approx $36,000) on the assumption the contract transfers to the buyer with no reassessment at the $8.5M price. A standard 1.2% reassessment would be approx $102,000. Verify the contract terms and pres</t>
   </si>
   <si>
     <t>PROPERTY</t>
@@ -303,16 +300,19 @@
     <t>Rent source</t>
   </si>
   <si>
-    <t>Allocated from published GRM (price / GRM) using LAAA bed weights</t>
-  </si>
-  <si>
-    <t>1 Bd / 1 Ba</t>
-  </si>
-  <si>
-    <t>2 Bd / 1 Ba</t>
-  </si>
-  <si>
-    <t>2 Bd / 2 Ba</t>
+    <t>2 Bd / 2 Ba townhouse  [953 #3 townhouse with private yard; market $6,000]</t>
+  </si>
+  <si>
+    <t>OM rent roll, current in-place rents (OM undated, sale comps through May 2026)</t>
+  </si>
+  <si>
+    <t>2 Bd / 1 Ba  [range $973-$4,187 occupied; includes 1 vacant unit carried a]</t>
+  </si>
+  <si>
+    <t>1 Bd / 1 Ba  [range $2,118-$3,960; market $4,000]</t>
+  </si>
+  <si>
+    <t>Studio  [range $1,989-$2,868; market $3,000]</t>
   </si>
   <si>
     <t>Total / weighted avg</t>
@@ -333,7 +333,7 @@
     <t>Scheduled gross rent</t>
   </si>
   <si>
-    <t>OM column: price / published GRM</t>
+    <t>OM column: OM stated current scheduled rent (OM undated, sale comps through May 2026); LAAA column: OM rent roll by unit type</t>
   </si>
   <si>
     <t>Other income (laundry, parking, RUBS)</t>
@@ -345,7 +345,7 @@
     <t>Vacancy &amp; credit loss</t>
   </si>
   <si>
-    <t>OM 3.0% (OM figure if extracted, else 3% assumed); LAAA per Assumptions</t>
+    <t>OM 3.0%; LAAA per Assumptions</t>
   </si>
   <si>
     <t>Effective gross income</t>
@@ -390,7 +390,7 @@
     <t>Utilities (water/sewer/trash/common electric &amp; gas)</t>
   </si>
   <si>
-    <t>per unit, by city</t>
+    <t>per unit, by city; OM utilities + water/sewer + gas/electric + trash combined</t>
   </si>
   <si>
     <t>Contract services (landscape, pest, cleaning)</t>
@@ -399,10 +399,10 @@
     <t>per unit</t>
   </si>
   <si>
-    <t>Admin / legal / licenses / rent registration</t>
-  </si>
-  <si>
-    <t>per unit; OM "other" items land here</t>
+    <t>Admin / legal / licenses / rent registration / other OM items</t>
+  </si>
+  <si>
+    <t>OM other items: General &amp; Administrative 4,232</t>
   </si>
   <si>
     <t>Replacement reserves</t>
@@ -411,7 +411,7 @@
     <t>Total operating expenses</t>
   </si>
   <si>
-    <t>OM line items not published. OM total IMPLIED = OM EGI - (price x published cap)</t>
+    <t>OM line items from OM (OM undated, sale comps through May 2026); basis: OM 'Current' column of Annualized Operating Data (p.16); broker figures, not owner actuals. Taxes $36,816 = current bill under the existing recorded Mills Act contract (OM says approx $36,000), NOT a reassessment at the $8.5M price. Management = 4.0% of EGI. Utilities is a single combined line. Market column identical except management $30,019 (4% of market EGI).; OM total 100,498</t>
   </si>
   <si>
     <t>Expenses per unit</t>
@@ -427,6 +427,9 @@
   </si>
   <si>
     <t>Net operating income</t>
+  </si>
+  <si>
+    <t>OM states NOI 498,774 / cap 5.87</t>
   </si>
   <si>
     <t>Cap rate on asking price</t>
@@ -475,12 +478,13 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="3">
+  <numFmts count="4">
     <numFmt numFmtId="164" formatCode="\$#,##0;\(\$#,##0\);&quot;-&quot;"/>
     <numFmt numFmtId="165" formatCode="\$#,##0.00"/>
     <numFmt numFmtId="166" formatCode="0.00&quot;x&quot;"/>
+    <numFmt numFmtId="167" formatCode="&quot;$&quot;#,##0;\(&quot;$&quot;#,##0\);&quot;-&quot;"/>
   </numFmts>
-  <fonts count="10" x14ac:knownFonts="1">
+  <fonts count="12" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -528,6 +532,7 @@
       <sz val="11"/>
       <color rgb="FFC00000"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
@@ -536,8 +541,21 @@
       <name val="Calibri"/>
     </font>
     <font>
+      <i/>
+      <sz val="9"/>
+      <color rgb="FF595959"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
       <b/>
       <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFC00000"/>
       <name val="Calibri"/>
     </font>
   </fonts>
@@ -565,7 +583,8 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFF9E5"/>
+        <fgColor rgb="FFFFF2CC"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
@@ -601,7 +620,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -625,12 +644,15 @@
     <xf numFmtId="0" fontId="8" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="167" fontId="0" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="3" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="3" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="8" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="164" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -663,7 +685,7 @@
         <xdr:cNvPr id="2" name="Image 1" descr="Picture">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{F827B8E8-8E4D-4057-955C-802B9DE9C906}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{563A888B-9CD0-465A-8C0F-42B87A3C429F}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -974,7 +996,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3E52B553-068D-4B59-B4BB-720C45DB1EC1}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B019AF4D-09FB-4554-8E7A-E8EBAA388E45}">
   <dimension ref="A1:C40"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -1343,7 +1365,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3E379121-9D05-4DEC-81A7-3A185AB4E2E4}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{49C2B0CD-8481-407E-A735-267058F38674}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
@@ -1571,116 +1593,116 @@
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>34</v>
+        <v>86</v>
       </c>
       <c r="B30" s="15">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C30" s="21">
-        <v>2316</v>
-      </c>
-      <c r="D30" s="8">
+        <v>5080</v>
+      </c>
+      <c r="D30" s="22">
         <f>B30*C30</f>
-        <v>9264</v>
-      </c>
-      <c r="E30" s="8">
+        <v>5080</v>
+      </c>
+      <c r="E30" s="22">
         <f>D30*12</f>
-        <v>111168</v>
-      </c>
-      <c r="F30" s="2" t="s">
-        <v>86</v>
+        <v>60960</v>
+      </c>
+      <c r="F30" s="23" t="s">
+        <v>87</v>
       </c>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
+        <v>88</v>
+      </c>
+      <c r="B31" s="15">
+        <v>4</v>
+      </c>
+      <c r="C31" s="21">
+        <v>3386</v>
+      </c>
+      <c r="D31" s="22">
+        <f>B31*C31</f>
+        <v>13544</v>
+      </c>
+      <c r="E31" s="22">
+        <f>D31*12</f>
+        <v>162528</v>
+      </c>
+      <c r="F31" s="23" t="s">
         <v>87</v>
-      </c>
-      <c r="B31" s="15">
-        <v>6</v>
-      </c>
-      <c r="C31" s="21">
-        <v>3308</v>
-      </c>
-      <c r="D31" s="8">
-        <f>B31*C31</f>
-        <v>19848</v>
-      </c>
-      <c r="E31" s="8">
-        <f>D31*12</f>
-        <v>238176</v>
-      </c>
-      <c r="F31" s="2" t="s">
-        <v>86</v>
       </c>
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="B32" s="15">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="C32" s="21">
-        <v>4466</v>
-      </c>
-      <c r="D32" s="8">
+        <v>3373</v>
+      </c>
+      <c r="D32" s="22">
         <f>B32*C32</f>
-        <v>17864</v>
-      </c>
-      <c r="E32" s="8">
+        <v>20238</v>
+      </c>
+      <c r="E32" s="22">
         <f>D32*12</f>
-        <v>214368</v>
-      </c>
-      <c r="F32" s="2" t="s">
-        <v>86</v>
+        <v>242856</v>
+      </c>
+      <c r="F32" s="23" t="s">
+        <v>87</v>
       </c>
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="B33" s="15">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C33" s="21">
-        <v>4466</v>
-      </c>
-      <c r="D33" s="8">
+        <v>2537</v>
+      </c>
+      <c r="D33" s="22">
         <f>B33*C33</f>
-        <v>4466</v>
-      </c>
-      <c r="E33" s="8">
+        <v>10148</v>
+      </c>
+      <c r="E33" s="22">
         <f>D33*12</f>
-        <v>53592</v>
-      </c>
-      <c r="F33" s="2" t="s">
-        <v>86</v>
+        <v>121776</v>
+      </c>
+      <c r="F33" s="23" t="s">
+        <v>87</v>
       </c>
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A34" s="22" t="s">
-        <v>90</v>
-      </c>
-      <c r="B34" s="23">
+      <c r="A34" s="24" t="s">
+        <v>91</v>
+      </c>
+      <c r="B34" s="25">
         <f>SUM(B30:B33)</f>
         <v>15</v>
       </c>
-      <c r="C34" s="24">
+      <c r="C34" s="26">
         <f>IFERROR(D34/B34,"")</f>
-        <v>3429.4666666666667</v>
-      </c>
-      <c r="D34" s="24">
+        <v>3267.3333333333335</v>
+      </c>
+      <c r="D34" s="26">
         <f>SUM(D30:D33)</f>
-        <v>51442</v>
-      </c>
-      <c r="E34" s="24">
+        <v>49010</v>
+      </c>
+      <c r="E34" s="26">
         <f>SUM(E30:E33)</f>
-        <v>617304</v>
+        <v>588120</v>
       </c>
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A36" s="13" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="B36" s="14"/>
       <c r="C36" s="14"/>
@@ -1689,90 +1711,90 @@
       <c r="F36" s="14"/>
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A37" s="25"/>
-      <c r="B37" s="25" t="s">
-        <v>92</v>
-      </c>
-      <c r="C37" s="25" t="s">
+      <c r="A37" s="27"/>
+      <c r="B37" s="27" t="s">
         <v>93</v>
       </c>
-      <c r="D37" s="25"/>
-      <c r="E37" s="25"/>
-      <c r="F37" s="25" t="s">
+      <c r="C37" s="27" t="s">
         <v>94</v>
+      </c>
+      <c r="D37" s="27"/>
+      <c r="E37" s="27"/>
+      <c r="F37" s="27" t="s">
+        <v>95</v>
       </c>
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>95</v>
-      </c>
-      <c r="B38" s="8">
-        <v>617283.95061728393</v>
+        <v>96</v>
+      </c>
+      <c r="B38" s="22">
+        <v>588114</v>
       </c>
       <c r="C38" s="8">
         <f>E34</f>
-        <v>617304</v>
+        <v>588120</v>
       </c>
       <c r="F38" s="2" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="B39" s="8">
-        <v>0</v>
+        <v>29340</v>
       </c>
       <c r="C39" s="4">
-        <v>0</v>
+        <v>29340</v>
       </c>
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A40" s="22" t="s">
-        <v>98</v>
+      <c r="A40" s="24" t="s">
+        <v>99</v>
       </c>
       <c r="B40" s="8">
         <f>B38+B39</f>
-        <v>617283.95061728393</v>
+        <v>617454</v>
       </c>
       <c r="C40" s="8">
         <f>C38+C39</f>
-        <v>617304</v>
+        <v>617460</v>
       </c>
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="B41" s="8">
         <f>-B38*0.03</f>
-        <v>-18518.518518518518</v>
+        <v>-17643.419999999998</v>
       </c>
       <c r="C41" s="8">
         <f>-C38*Assumptions!$B$3</f>
-        <v>-18519.12</v>
+        <v>-17643.599999999999</v>
       </c>
       <c r="F41" s="2" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A42" s="22" t="s">
-        <v>101</v>
-      </c>
-      <c r="B42" s="24">
+      <c r="A42" s="24" t="s">
+        <v>102</v>
+      </c>
+      <c r="B42" s="26">
         <f>B40+B41</f>
-        <v>598765.43209876539</v>
-      </c>
-      <c r="C42" s="24">
+        <v>599810.57999999996</v>
+      </c>
+      <c r="C42" s="26">
         <f>C40+C41</f>
-        <v>598784.88</v>
+        <v>599816.4</v>
       </c>
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A44" s="13" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="B44" s="14"/>
       <c r="C44" s="14"/>
@@ -1781,182 +1803,196 @@
       <c r="F44" s="14"/>
     </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A45" s="25" t="s">
-        <v>103</v>
-      </c>
-      <c r="B45" s="25" t="s">
-        <v>92</v>
-      </c>
-      <c r="C45" s="25" t="s">
+      <c r="A45" s="27" t="s">
         <v>104</v>
       </c>
-      <c r="D45" s="25" t="s">
+      <c r="B45" s="27" t="s">
         <v>93</v>
       </c>
-      <c r="E45" s="25" t="s">
+      <c r="C45" s="27" t="s">
         <v>105</v>
       </c>
-      <c r="F45" s="25" t="s">
+      <c r="D45" s="27" t="s">
         <v>94</v>
+      </c>
+      <c r="E45" s="27" t="s">
+        <v>106</v>
+      </c>
+      <c r="F45" s="27" t="s">
+        <v>95</v>
       </c>
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>106</v>
-      </c>
-      <c r="B46" s="8"/>
+        <v>107</v>
+      </c>
+      <c r="B46" s="22">
+        <v>36816</v>
+      </c>
       <c r="C46" s="8">
         <f>B22*Assumptions!$B$16</f>
         <v>97750</v>
       </c>
-      <c r="D46" s="26">
+      <c r="D46" s="28">
         <f>C46</f>
         <v>97750</v>
       </c>
-      <c r="E46" s="8" t="str">
+      <c r="E46" s="8">
         <f t="shared" ref="E46:E54" si="0">IF(ISNUMBER(B46),D46-B46,"")</f>
-        <v/>
+        <v>60934</v>
       </c>
       <c r="F46" s="2" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
     </row>
     <row r="47" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>108</v>
-      </c>
-      <c r="B47" s="8"/>
+        <v>109</v>
+      </c>
+      <c r="B47" s="22">
+        <v>14578</v>
+      </c>
       <c r="C47" s="8">
         <f>B7*Assumptions!$B$5+B8*Assumptions!$B$6</f>
         <v>14850</v>
       </c>
-      <c r="D47" s="26">
+      <c r="D47" s="28">
         <f t="shared" ref="D47:D53" si="1">IF(ISNUMBER(B47),MAX(B47,C47),C47)</f>
         <v>14850</v>
       </c>
-      <c r="E47" s="8" t="str">
+      <c r="E47" s="8">
         <f t="shared" si="0"/>
-        <v/>
+        <v>272</v>
       </c>
       <c r="F47" s="2" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
     </row>
     <row r="48" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>110</v>
-      </c>
-      <c r="B48" s="8"/>
+        <v>111</v>
+      </c>
+      <c r="B48" s="22">
+        <v>23971</v>
+      </c>
       <c r="C48" s="8">
         <f>C42*Assumptions!$B$4</f>
-        <v>29939.244000000002</v>
-      </c>
-      <c r="D48" s="26">
+        <v>29990.820000000003</v>
+      </c>
+      <c r="D48" s="28">
         <f t="shared" si="1"/>
-        <v>29939.244000000002</v>
-      </c>
-      <c r="E48" s="8" t="str">
+        <v>29990.820000000003</v>
+      </c>
+      <c r="E48" s="8">
         <f t="shared" si="0"/>
-        <v/>
+        <v>6019.8200000000033</v>
       </c>
       <c r="F48" s="2" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
     </row>
     <row r="49" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>112</v>
-      </c>
-      <c r="B49" s="8"/>
+        <v>113</v>
+      </c>
+      <c r="B49" s="22">
+        <v>6000</v>
+      </c>
       <c r="C49" s="8">
         <f>B7*Assumptions!$B$7</f>
         <v>18000</v>
       </c>
-      <c r="D49" s="26">
+      <c r="D49" s="28">
         <f t="shared" si="1"/>
         <v>18000</v>
       </c>
-      <c r="E49" s="8" t="str">
+      <c r="E49" s="8">
         <f t="shared" si="0"/>
-        <v/>
+        <v>12000</v>
       </c>
       <c r="F49" s="2" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
     </row>
     <row r="50" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>114</v>
-      </c>
-      <c r="B50" s="8"/>
+        <v>115</v>
+      </c>
+      <c r="B50" s="22">
+        <v>12981</v>
+      </c>
       <c r="C50" s="8">
         <f>B7*Assumptions!$B$10</f>
         <v>27000</v>
       </c>
-      <c r="D50" s="26">
+      <c r="D50" s="28">
         <f t="shared" si="1"/>
         <v>27000</v>
       </c>
-      <c r="E50" s="8" t="str">
+      <c r="E50" s="8">
         <f t="shared" si="0"/>
-        <v/>
+        <v>14019</v>
       </c>
       <c r="F50" s="2" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
     </row>
     <row r="51" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>116</v>
-      </c>
-      <c r="B51" s="8"/>
+        <v>117</v>
+      </c>
+      <c r="B51" s="22">
+        <v>1920</v>
+      </c>
       <c r="C51" s="8">
         <f>B7*Assumptions!$B$12</f>
         <v>6000</v>
       </c>
-      <c r="D51" s="26">
+      <c r="D51" s="28">
         <f t="shared" si="1"/>
         <v>6000</v>
       </c>
-      <c r="E51" s="8" t="str">
+      <c r="E51" s="8">
         <f t="shared" si="0"/>
-        <v/>
+        <v>4080</v>
       </c>
       <c r="F51" s="2" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
     </row>
     <row r="52" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>118</v>
-      </c>
-      <c r="B52" s="8"/>
+        <v>119</v>
+      </c>
+      <c r="B52" s="22">
+        <v>4232</v>
+      </c>
       <c r="C52" s="8">
         <f>B7*Assumptions!$B$13</f>
         <v>3750</v>
       </c>
-      <c r="D52" s="26">
+      <c r="D52" s="28">
         <f t="shared" si="1"/>
-        <v>3750</v>
-      </c>
-      <c r="E52" s="8" t="str">
+        <v>4232</v>
+      </c>
+      <c r="E52" s="8">
         <f t="shared" si="0"/>
-        <v/>
+        <v>0</v>
       </c>
       <c r="F52" s="2" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
     </row>
     <row r="53" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>120</v>
-      </c>
-      <c r="B53" s="8"/>
+        <v>121</v>
+      </c>
+      <c r="B53" s="22"/>
       <c r="C53" s="8">
         <f>B7*Assumptions!$B$14</f>
         <v>4500</v>
       </c>
-      <c r="D53" s="26">
+      <c r="D53" s="28">
         <f t="shared" si="1"/>
         <v>4500</v>
       </c>
@@ -1965,79 +2001,79 @@
         <v/>
       </c>
       <c r="F53" s="2" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
     </row>
     <row r="54" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A54" s="22" t="s">
-        <v>121</v>
-      </c>
-      <c r="B54" s="24">
-        <f>B42-B22*B25</f>
-        <v>85365.432098765392</v>
-      </c>
-      <c r="C54" s="24">
+      <c r="A54" s="24" t="s">
+        <v>122</v>
+      </c>
+      <c r="B54" s="26">
+        <f>SUM(B46:B53)</f>
+        <v>100498</v>
+      </c>
+      <c r="C54" s="26">
         <f>SUM(C46:C53)</f>
-        <v>201789.24400000001</v>
-      </c>
-      <c r="D54" s="24">
+        <v>201840.82</v>
+      </c>
+      <c r="D54" s="26">
         <f>SUM(D46:D53)</f>
-        <v>201789.24400000001</v>
-      </c>
-      <c r="E54" s="24">
+        <v>202322.82</v>
+      </c>
+      <c r="E54" s="26">
         <f t="shared" si="0"/>
-        <v>116423.81190123461</v>
+        <v>101824.82</v>
       </c>
       <c r="F54" s="2" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
     </row>
     <row r="55" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="B55" s="8">
         <f>IFERROR(B54/B7,"")</f>
-        <v>5691.0288065843597</v>
+        <v>6699.8666666666668</v>
       </c>
       <c r="C55" s="8">
         <f>IFERROR(C54/B7,"")</f>
-        <v>13452.616266666668</v>
+        <v>13456.054666666667</v>
       </c>
       <c r="D55" s="8">
         <f>IFERROR(D54/B7,"")</f>
-        <v>13452.616266666668</v>
+        <v>13488.188</v>
       </c>
     </row>
     <row r="56" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="B56" s="18">
         <f>IFERROR(B54/B42,"")</f>
-        <v>0.14256907216494841</v>
+        <v>0.1675495620634101</v>
       </c>
       <c r="C56" s="18">
         <f>IFERROR(C54/C42,"")</f>
-        <v>0.33699789480322218</v>
+        <v>0.33650433699378679</v>
       </c>
       <c r="D56" s="18">
         <f>IF(C38&gt;0,IFERROR(D54/C42,""),"")</f>
-        <v>0.33699789480322218</v>
+        <v>0.33730791622236406</v>
       </c>
     </row>
     <row r="57" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A57" s="22" t="s">
-        <v>125</v>
-      </c>
-      <c r="B57" s="12" t="str">
+      <c r="A57" s="24" t="s">
+        <v>126</v>
+      </c>
+      <c r="B57" s="29" t="str">
         <f>IF(ISNUMBER(B54),IF(D54&gt;B54*(1+Assumptions!$B$24),"OM EXPENSES LIGHT","OM expenses reasonable"),"OM expenses not published")</f>
         <v>OM EXPENSES LIGHT</v>
       </c>
     </row>
     <row r="59" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A59" s="13" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="B59" s="14"/>
       <c r="C59" s="14"/>
@@ -2046,77 +2082,80 @@
       <c r="F59" s="14"/>
     </row>
     <row r="60" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A60" s="25"/>
-      <c r="B60" s="25" t="s">
-        <v>92</v>
-      </c>
-      <c r="C60" s="25" t="s">
+      <c r="A60" s="27"/>
+      <c r="B60" s="27" t="s">
         <v>93</v>
       </c>
-      <c r="D60" s="25"/>
-      <c r="E60" s="25"/>
-      <c r="F60" s="25" t="s">
+      <c r="C60" s="27" t="s">
         <v>94</v>
       </c>
+      <c r="D60" s="27"/>
+      <c r="E60" s="27"/>
+      <c r="F60" s="27" t="s">
+        <v>95</v>
+      </c>
     </row>
     <row r="61" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A61" s="22" t="s">
-        <v>127</v>
-      </c>
-      <c r="B61" s="24">
+      <c r="A61" s="24" t="s">
+        <v>128</v>
+      </c>
+      <c r="B61" s="26">
         <f>B42-B54</f>
-        <v>513400</v>
-      </c>
-      <c r="C61" s="24">
+        <v>499312.57999999996</v>
+      </c>
+      <c r="C61" s="26">
         <f>IF(C38&gt;0,C42-D54,"")</f>
-        <v>396995.636</v>
+        <v>397493.58</v>
+      </c>
+      <c r="F61" t="s">
+        <v>129</v>
       </c>
     </row>
     <row r="62" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A62" s="22" t="s">
-        <v>128</v>
+      <c r="A62" s="24" t="s">
+        <v>130</v>
       </c>
       <c r="B62" s="18">
         <f>IFERROR(B61/B22,"")</f>
-        <v>6.0400000000000002E-2</v>
+        <v>5.8742656470588232E-2</v>
       </c>
       <c r="C62" s="18">
         <f>IF(C61="","",IFERROR(C61/B22,""))</f>
-        <v>4.6705368941176467E-2</v>
+        <v>4.6763950588235299E-2</v>
       </c>
       <c r="F62" s="2" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
     </row>
     <row r="63" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="B63" s="19">
         <f>IFERROR(B22/B38,"")</f>
-        <v>13.77</v>
+        <v>14.452980204518171</v>
       </c>
       <c r="C63" s="19">
         <f>IF(C38&gt;0,IFERROR(B22/C38,""),"")</f>
-        <v>13.769552764926194</v>
+        <v>14.452832755220022</v>
       </c>
     </row>
     <row r="64" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="B64" s="8">
         <f>IFERROR(B61/B7,"")</f>
-        <v>34226.666666666664</v>
+        <v>33287.505333333327</v>
       </c>
       <c r="C64" s="8">
         <f>IF(C61="","",IFERROR(C61/B7,""))</f>
-        <v>26466.375733333334</v>
+        <v>26499.572</v>
       </c>
     </row>
     <row r="66" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A66" s="13" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="B66" s="14"/>
       <c r="C66" s="14"/>
@@ -2126,7 +2165,7 @@
     </row>
     <row r="67" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="B67" s="8">
         <f>IFERROR(B22*Assumptions!$B$20,"")</f>
@@ -2135,79 +2174,78 @@
     </row>
     <row r="68" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="B68" s="8">
         <f>IF(C61="","",IFERROR(PV(Assumptions!$B$22/12,Assumptions!$B$23*12,-C61/Assumptions!$B$21/12),""))</f>
-        <v>4298462.949387311</v>
+        <v>4303854.4288918097</v>
       </c>
     </row>
     <row r="69" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A69" s="22" t="s">
-        <v>135</v>
+      <c r="A69" s="24" t="s">
+        <v>137</v>
       </c>
       <c r="B69" s="8">
         <f>IFERROR(MIN(B67,B68),"")</f>
-        <v>4298462.949387311</v>
+        <v>4303854.4288918097</v>
       </c>
     </row>
     <row r="70" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="B70" s="8">
         <f>IFERROR(B22-B69,"")</f>
-        <v>4201537.050612689</v>
+        <v>4196145.5711081903</v>
       </c>
     </row>
     <row r="71" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="B71" s="8">
         <f>IFERROR(-PMT(Assumptions!$B$22/12,Assumptions!$B$23*12,B69)*12,"")</f>
-        <v>317596.50879999902</v>
+        <v>317994.86399999895</v>
       </c>
     </row>
     <row r="72" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="B72" s="19">
         <f>IFERROR(C61/B71,"")</f>
-        <v>1.2500000000000038</v>
+        <v>1.2500000000000042</v>
       </c>
     </row>
     <row r="73" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="B73" s="8">
         <f>IFERROR(C61-B71,"")</f>
-        <v>79399.127200000978</v>
+        <v>79498.716000001063</v>
       </c>
     </row>
     <row r="74" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="B74" s="18">
         <f>IFERROR(B73/B70,"")</f>
-        <v>1.8897638231804383E-2</v>
+        <v>1.8945652540601845E-2</v>
       </c>
     </row>
     <row r="76" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A76" s="2" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="A3" r:id="rId1" xr:uid="{37EADA75-7FE2-4D66-8757-7CBEBF0CE64F}"/>
+    <hyperlink ref="A3" r:id="rId1" xr:uid="{8FE4F189-1C69-4E72-BF08-644CFBA9F958}"/>
   </hyperlinks>
-  <printOptions horizontalCentered="1"/>
-  <pageMargins left="0.25" right="0.25" top="0.25" bottom="0.25" header="0.5" footer="0.5"/>
-  <pageSetup scale="50" orientation="landscape" r:id="rId2"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" r:id="rId2"/>
   <drawing r:id="rId3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
947-953 11th St: LAAA column keeps Mills Act taxes ($36,816), not reassessed at price
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/files/03-947-953-11th-st.xlsx
+++ b/files/03-947-953-11th-st.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\iniculete\LAAA-Deploys\onmarket\files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{93D6BE28-8CD9-42FE-8D18-22C275D06059}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{80E3B3E7-A0E3-4D40-9574-C040CD65D2F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{26B3E24F-726B-438B-AD7A-01605760F0D5}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{FE5559C7-D0FB-49B9-BD91-BA3936FB4F19}"/>
   </bookViews>
   <sheets>
     <sheet name="Assumptions" sheetId="1" r:id="rId1"/>
@@ -195,7 +195,7 @@
     <t>Data pulled 9/17/2026 from LoopNet public listing + rent roll and expenses read from the listing broker's OM (Equity Union Commercial (The Appel Group), Eliyahu Appel, undated, sale comps through May 2026)</t>
   </si>
   <si>
-    <t>NOTE: 80% occupied per LoopNet | OM: Mills Act: existing recorded Mills Act contract; OM carries property taxes at $36,816 (current bill approx $36,000) on the assumption the contract transfers to the buyer with no reassessment at the $8.5M price. A standard 1.2% reassessment would be approx $102,000. Verify the contract terms and pres</t>
+    <t>NOTE: 80% occupied per LoopNet | OM: Mills Act: existing recorded Mills Act contract transfers to the buyer, so property taxes stay at the current $36,816 (OM says approx $36,000) with no reassessment at the $8.5M price; LAAA column uses this figure per Filip 9/17. Verify the contract terms and preservation obligations in escrow.; Vaca</t>
   </si>
   <si>
     <t>PROPERTY</t>
@@ -363,10 +363,10 @@
     <t>Delta vs OM</t>
   </si>
   <si>
-    <t>Property taxes (reassessed at price)</t>
-  </si>
-  <si>
-    <t>Santa Monica rate x asking price; always reassessed, never MAX</t>
+    <t>Property taxes (Mills Act, not reassessed)</t>
+  </si>
+  <si>
+    <t>Mills Act: existing recorded contract transfers with the property; taxes NOT reassessed at price (Filip 9/17). OM figure used in the LAAA column.</t>
   </si>
   <si>
     <t>Insurance</t>
@@ -620,7 +620,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -651,6 +651,7 @@
     <xf numFmtId="3" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="8" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="167" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="164" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
@@ -685,7 +686,7 @@
         <xdr:cNvPr id="2" name="Image 1" descr="Picture">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{563A888B-9CD0-465A-8C0F-42B87A3C429F}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{3AD417A1-A97A-4504-AD29-9EF324D3924A}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -996,7 +997,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B019AF4D-09FB-4554-8E7A-E8EBAA388E45}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{467128BD-5A2E-48BB-8B24-CEAAA4080EBB}">
   <dimension ref="A1:C40"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -1365,7 +1366,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{49C2B0CD-8481-407E-A735-267058F38674}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6A6D9DAD-7731-49F2-A6EE-83F1AD297BB3}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
@@ -1834,12 +1835,11 @@
         <v>97750</v>
       </c>
       <c r="D46" s="28">
-        <f>C46</f>
-        <v>97750</v>
+        <v>36816</v>
       </c>
       <c r="E46" s="8">
         <f t="shared" ref="E46:E54" si="0">IF(ISNUMBER(B46),D46-B46,"")</f>
-        <v>60934</v>
+        <v>0</v>
       </c>
       <c r="F46" s="2" t="s">
         <v>108</v>
@@ -1856,7 +1856,7 @@
         <f>B7*Assumptions!$B$5+B8*Assumptions!$B$6</f>
         <v>14850</v>
       </c>
-      <c r="D47" s="28">
+      <c r="D47" s="29">
         <f t="shared" ref="D47:D53" si="1">IF(ISNUMBER(B47),MAX(B47,C47),C47)</f>
         <v>14850</v>
       </c>
@@ -1879,7 +1879,7 @@
         <f>C42*Assumptions!$B$4</f>
         <v>29990.820000000003</v>
       </c>
-      <c r="D48" s="28">
+      <c r="D48" s="29">
         <f t="shared" si="1"/>
         <v>29990.820000000003</v>
       </c>
@@ -1902,7 +1902,7 @@
         <f>B7*Assumptions!$B$7</f>
         <v>18000</v>
       </c>
-      <c r="D49" s="28">
+      <c r="D49" s="29">
         <f t="shared" si="1"/>
         <v>18000</v>
       </c>
@@ -1925,7 +1925,7 @@
         <f>B7*Assumptions!$B$10</f>
         <v>27000</v>
       </c>
-      <c r="D50" s="28">
+      <c r="D50" s="29">
         <f t="shared" si="1"/>
         <v>27000</v>
       </c>
@@ -1948,7 +1948,7 @@
         <f>B7*Assumptions!$B$12</f>
         <v>6000</v>
       </c>
-      <c r="D51" s="28">
+      <c r="D51" s="29">
         <f t="shared" si="1"/>
         <v>6000</v>
       </c>
@@ -1971,7 +1971,7 @@
         <f>B7*Assumptions!$B$13</f>
         <v>3750</v>
       </c>
-      <c r="D52" s="28">
+      <c r="D52" s="29">
         <f t="shared" si="1"/>
         <v>4232</v>
       </c>
@@ -1992,7 +1992,7 @@
         <f>B7*Assumptions!$B$14</f>
         <v>4500</v>
       </c>
-      <c r="D53" s="28">
+      <c r="D53" s="29">
         <f t="shared" si="1"/>
         <v>4500</v>
       </c>
@@ -2018,11 +2018,11 @@
       </c>
       <c r="D54" s="26">
         <f>SUM(D46:D53)</f>
-        <v>202322.82</v>
+        <v>141388.82</v>
       </c>
       <c r="E54" s="26">
         <f t="shared" si="0"/>
-        <v>101824.82</v>
+        <v>40890.820000000007</v>
       </c>
       <c r="F54" s="2" t="s">
         <v>123</v>
@@ -2042,7 +2042,7 @@
       </c>
       <c r="D55" s="8">
         <f>IFERROR(D54/B7,"")</f>
-        <v>13488.188</v>
+        <v>9425.9213333333337</v>
       </c>
     </row>
     <row r="56" spans="1:6" x14ac:dyDescent="0.25">
@@ -2059,14 +2059,14 @@
       </c>
       <c r="D56" s="18">
         <f>IF(C38&gt;0,IFERROR(D54/C42,""),"")</f>
-        <v>0.33730791622236406</v>
+        <v>0.23572016370342658</v>
       </c>
     </row>
     <row r="57" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A57" s="24" t="s">
         <v>126</v>
       </c>
-      <c r="B57" s="29" t="str">
+      <c r="B57" s="30" t="str">
         <f>IF(ISNUMBER(B54),IF(D54&gt;B54*(1+Assumptions!$B$24),"OM EXPENSES LIGHT","OM expenses reasonable"),"OM expenses not published")</f>
         <v>OM EXPENSES LIGHT</v>
       </c>
@@ -2105,7 +2105,7 @@
       </c>
       <c r="C61" s="26">
         <f>IF(C38&gt;0,C42-D54,"")</f>
-        <v>397493.58</v>
+        <v>458427.58</v>
       </c>
       <c r="F61" t="s">
         <v>129</v>
@@ -2121,7 +2121,7 @@
       </c>
       <c r="C62" s="18">
         <f>IF(C61="","",IFERROR(C61/B22,""))</f>
-        <v>4.6763950588235299E-2</v>
+        <v>5.3932656470588237E-2</v>
       </c>
       <c r="F62" s="2" t="s">
         <v>131</v>
@@ -2150,7 +2150,7 @@
       </c>
       <c r="C64" s="8">
         <f>IF(C61="","",IFERROR(C61/B7,""))</f>
-        <v>26499.572</v>
+        <v>30561.838666666667</v>
       </c>
     </row>
     <row r="66" spans="1:6" x14ac:dyDescent="0.25">
@@ -2178,7 +2178,7 @@
       </c>
       <c r="B68" s="8">
         <f>IF(C61="","",IFERROR(PV(Assumptions!$B$22/12,Assumptions!$B$23*12,-C61/Assumptions!$B$21/12),""))</f>
-        <v>4303854.4288918097</v>
+        <v>4963616.1935223071</v>
       </c>
     </row>
     <row r="69" spans="1:6" x14ac:dyDescent="0.25">
@@ -2187,7 +2187,7 @@
       </c>
       <c r="B69" s="8">
         <f>IFERROR(MIN(B67,B68),"")</f>
-        <v>4303854.4288918097</v>
+        <v>4963616.1935223071</v>
       </c>
     </row>
     <row r="70" spans="1:6" x14ac:dyDescent="0.25">
@@ -2196,7 +2196,7 @@
       </c>
       <c r="B70" s="8">
         <f>IFERROR(B22-B69,"")</f>
-        <v>4196145.5711081903</v>
+        <v>3536383.8064776929</v>
       </c>
     </row>
     <row r="71" spans="1:6" x14ac:dyDescent="0.25">
@@ -2205,7 +2205,7 @@
       </c>
       <c r="B71" s="8">
         <f>IFERROR(-PMT(Assumptions!$B$22/12,Assumptions!$B$23*12,B69)*12,"")</f>
-        <v>317994.86399999895</v>
+        <v>366742.06399999885</v>
       </c>
     </row>
     <row r="72" spans="1:6" x14ac:dyDescent="0.25">
@@ -2214,7 +2214,7 @@
       </c>
       <c r="B72" s="19">
         <f>IFERROR(C61/B71,"")</f>
-        <v>1.2500000000000042</v>
+        <v>1.250000000000004</v>
       </c>
     </row>
     <row r="73" spans="1:6" x14ac:dyDescent="0.25">
@@ -2223,7 +2223,7 @@
       </c>
       <c r="B73" s="8">
         <f>IFERROR(C61-B71,"")</f>
-        <v>79498.716000001063</v>
+        <v>91685.516000001167</v>
       </c>
     </row>
     <row r="74" spans="1:6" x14ac:dyDescent="0.25">
@@ -2232,7 +2232,7 @@
       </c>
       <c r="B74" s="18">
         <f>IFERROR(B73/B70,"")</f>
-        <v>1.8945652540601845E-2</v>
+        <v>2.5926347652666618E-2</v>
       </c>
     </row>
     <row r="76" spans="1:6" x14ac:dyDescent="0.25">
@@ -2242,7 +2242,7 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="A3" r:id="rId1" xr:uid="{8FE4F189-1C69-4E72-BF08-644CFBA9F958}"/>
+    <hyperlink ref="A3" r:id="rId1" xr:uid="{5FEB6DD2-739E-4711-A1E6-E98D4DC47C44}"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" r:id="rId2"/>

</xml_diff>